<commit_message>
other name to correct
</commit_message>
<xml_diff>
--- a/tools/excel/tisax/tisax-v5.1.xlsx
+++ b/tools/excel/tisax/tisax-v5.1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/titouanamelinedecadeville/Documents/ciso-assistant-community/tools/excel/tisax/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57A01F43-2086-984C-9991-940D4FD5ADB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0F82D25-0208-0F4D-A63D-FA37A33ADCDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="library_meta" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="818" uniqueCount="393">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="818" uniqueCount="392">
   <si>
     <t>type</t>
   </si>
@@ -59,9 +59,6 @@
   </si>
   <si>
     <t>name</t>
-  </si>
-  <si>
-    <t>Trusted Information Security Assessment Exchange</t>
   </si>
   <si>
     <t>description</t>
@@ -1952,39 +1949,39 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" t="s">
         <v>12</v>
-      </c>
-      <c r="B7" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
         <v>14</v>
-      </c>
-      <c r="B8" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" t="s">
         <v>16</v>
-      </c>
-      <c r="B9" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" t="s">
         <v>18</v>
-      </c>
-      <c r="B10" t="s">
-        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -2002,15 +1999,15 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" t="s">
         <v>21</v>
-      </c>
-      <c r="B2" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -2018,7 +2015,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -2034,47 +2031,47 @@
         <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>391</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" t="s">
         <v>12</v>
-      </c>
-      <c r="B6" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" t="s">
         <v>24</v>
-      </c>
-      <c r="B7" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" t="s">
         <v>26</v>
-      </c>
-      <c r="B8" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" t="s">
         <v>28</v>
-      </c>
-      <c r="B9" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" t="s">
         <v>30</v>
-      </c>
-      <c r="B10" t="s">
-        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -2089,10 +2086,10 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" t="s">
         <v>32</v>
-      </c>
-      <c r="B1" t="s">
-        <v>33</v>
       </c>
       <c r="C1" t="s">
         <v>8</v>
@@ -2101,10 +2098,10 @@
         <v>10</v>
       </c>
       <c r="E1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -2115,7 +2112,7 @@
         <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -2123,10 +2120,10 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E3" t="s">
         <v>35</v>
-      </c>
-      <c r="E3" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -2134,44 +2131,44 @@
         <v>3</v>
       </c>
       <c r="C4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E4" t="s">
         <v>37</v>
-      </c>
-      <c r="E4" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B5">
         <v>4</v>
       </c>
       <c r="D5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E5" t="s">
         <v>40</v>
       </c>
-      <c r="E5" t="s">
-        <v>41</v>
-      </c>
       <c r="F5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B6">
         <v>4</v>
       </c>
       <c r="D6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E6" t="s">
         <v>43</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>44</v>
-      </c>
-      <c r="F6" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -2179,10 +2176,10 @@
         <v>2</v>
       </c>
       <c r="C7" t="s">
+        <v>45</v>
+      </c>
+      <c r="E7" t="s">
         <v>46</v>
-      </c>
-      <c r="E7" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -2190,27 +2187,27 @@
         <v>3</v>
       </c>
       <c r="C8" t="s">
+        <v>47</v>
+      </c>
+      <c r="E8" t="s">
         <v>48</v>
-      </c>
-      <c r="E8" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B9">
         <v>4</v>
       </c>
       <c r="D9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -2218,61 +2215,61 @@
         <v>3</v>
       </c>
       <c r="C10" t="s">
+        <v>50</v>
+      </c>
+      <c r="E10" t="s">
         <v>51</v>
-      </c>
-      <c r="E10" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B11">
         <v>4</v>
       </c>
       <c r="D11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B12">
         <v>4</v>
       </c>
       <c r="D12" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E12" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F12" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B13">
         <v>4</v>
       </c>
       <c r="D13" t="s">
+        <v>54</v>
+      </c>
+      <c r="E13" t="s">
         <v>55</v>
       </c>
-      <c r="E13" t="s">
+      <c r="F13" t="s">
         <v>56</v>
-      </c>
-      <c r="F13" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -2280,61 +2277,61 @@
         <v>3</v>
       </c>
       <c r="C14" t="s">
+        <v>57</v>
+      </c>
+      <c r="E14" t="s">
         <v>58</v>
-      </c>
-      <c r="E14" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B15">
         <v>4</v>
       </c>
       <c r="D15" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E15" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F15" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B16">
         <v>4</v>
       </c>
       <c r="D16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E16" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F16" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B17">
         <v>4</v>
       </c>
       <c r="D17" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E17" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F17" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
@@ -2342,61 +2339,61 @@
         <v>3</v>
       </c>
       <c r="C18" t="s">
+        <v>62</v>
+      </c>
+      <c r="E18" t="s">
         <v>63</v>
-      </c>
-      <c r="E18" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B19">
         <v>4</v>
       </c>
       <c r="D19" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E19" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F19" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B20">
         <v>4</v>
       </c>
       <c r="D20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E20" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F20" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B21">
         <v>4</v>
       </c>
       <c r="D21" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E21" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F21" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
@@ -2404,10 +2401,10 @@
         <v>2</v>
       </c>
       <c r="C22" t="s">
+        <v>67</v>
+      </c>
+      <c r="E22" t="s">
         <v>68</v>
-      </c>
-      <c r="E22" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
@@ -2415,44 +2412,44 @@
         <v>3</v>
       </c>
       <c r="C23" t="s">
+        <v>69</v>
+      </c>
+      <c r="E23" t="s">
         <v>70</v>
-      </c>
-      <c r="E23" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B24">
         <v>4</v>
       </c>
       <c r="D24" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E24" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F24" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B25">
         <v>4</v>
       </c>
       <c r="D25" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E25" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F25" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
@@ -2460,44 +2457,44 @@
         <v>3</v>
       </c>
       <c r="C26" t="s">
+        <v>73</v>
+      </c>
+      <c r="E26" t="s">
         <v>74</v>
-      </c>
-      <c r="E26" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B27">
         <v>4</v>
       </c>
       <c r="D27" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E27" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F27" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B28">
         <v>4</v>
       </c>
       <c r="D28" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E28" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F28" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
@@ -2505,44 +2502,44 @@
         <v>3</v>
       </c>
       <c r="C29" t="s">
+        <v>77</v>
+      </c>
+      <c r="E29" t="s">
         <v>78</v>
-      </c>
-      <c r="E29" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B30">
         <v>4</v>
       </c>
       <c r="D30" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E30" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F30" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B31">
         <v>4</v>
       </c>
       <c r="D31" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E31" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F31" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.2">
@@ -2550,10 +2547,10 @@
         <v>2</v>
       </c>
       <c r="C32" t="s">
+        <v>81</v>
+      </c>
+      <c r="E32" t="s">
         <v>82</v>
-      </c>
-      <c r="E32" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.2">
@@ -2561,44 +2558,44 @@
         <v>3</v>
       </c>
       <c r="C33" t="s">
+        <v>83</v>
+      </c>
+      <c r="E33" t="s">
         <v>84</v>
-      </c>
-      <c r="E33" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B34">
         <v>4</v>
       </c>
       <c r="D34" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E34" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F34" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B35">
         <v>4</v>
       </c>
       <c r="D35" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E35" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F35" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
@@ -2606,10 +2603,10 @@
         <v>2</v>
       </c>
       <c r="C36" t="s">
+        <v>87</v>
+      </c>
+      <c r="E36" t="s">
         <v>88</v>
-      </c>
-      <c r="E36" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.2">
@@ -2617,44 +2614,44 @@
         <v>3</v>
       </c>
       <c r="C37" t="s">
+        <v>89</v>
+      </c>
+      <c r="E37" t="s">
         <v>90</v>
-      </c>
-      <c r="E37" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B38">
         <v>4</v>
       </c>
       <c r="D38" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E38" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F38" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B39">
         <v>4</v>
       </c>
       <c r="D39" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E39" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F39" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.2">
@@ -2662,44 +2659,44 @@
         <v>3</v>
       </c>
       <c r="C40" t="s">
+        <v>93</v>
+      </c>
+      <c r="E40" t="s">
         <v>94</v>
-      </c>
-      <c r="E40" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B41">
         <v>4</v>
       </c>
       <c r="D41" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E41" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F41" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B42">
         <v>4</v>
       </c>
       <c r="D42" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E42" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F42" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.2">
@@ -2707,10 +2704,10 @@
         <v>2</v>
       </c>
       <c r="C43" t="s">
+        <v>97</v>
+      </c>
+      <c r="E43" t="s">
         <v>98</v>
-      </c>
-      <c r="E43" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.2">
@@ -2718,61 +2715,61 @@
         <v>3</v>
       </c>
       <c r="C44" t="s">
+        <v>99</v>
+      </c>
+      <c r="E44" t="s">
         <v>100</v>
-      </c>
-      <c r="E44" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B45">
         <v>4</v>
       </c>
       <c r="D45" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E45" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F45" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B46">
         <v>4</v>
       </c>
       <c r="D46" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E46" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F46" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B47">
         <v>4</v>
       </c>
       <c r="D47" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E47" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F47" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.2">
@@ -2780,10 +2777,10 @@
         <v>1</v>
       </c>
       <c r="C48" t="s">
+        <v>104</v>
+      </c>
+      <c r="D48" t="s">
         <v>105</v>
-      </c>
-      <c r="D48" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.2">
@@ -2791,44 +2788,44 @@
         <v>2</v>
       </c>
       <c r="C49" t="s">
+        <v>106</v>
+      </c>
+      <c r="E49" t="s">
         <v>107</v>
-      </c>
-      <c r="E49" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B50">
         <v>3</v>
       </c>
       <c r="D50" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E50" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F50" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B51">
         <v>3</v>
       </c>
       <c r="D51" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E51" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F51" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.2">
@@ -2836,44 +2833,44 @@
         <v>2</v>
       </c>
       <c r="C52" t="s">
+        <v>110</v>
+      </c>
+      <c r="E52" t="s">
         <v>111</v>
-      </c>
-      <c r="E52" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B53">
         <v>3</v>
       </c>
       <c r="D53" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E53" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F53" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B54">
         <v>3</v>
       </c>
       <c r="D54" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E54" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F54" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.2">
@@ -2881,44 +2878,44 @@
         <v>2</v>
       </c>
       <c r="C55" t="s">
+        <v>114</v>
+      </c>
+      <c r="E55" t="s">
         <v>115</v>
-      </c>
-      <c r="E55" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B56">
         <v>3</v>
       </c>
       <c r="D56" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E56" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F56" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B57">
         <v>3</v>
       </c>
       <c r="D57" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E57" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F57" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.2">
@@ -2926,61 +2923,61 @@
         <v>2</v>
       </c>
       <c r="C58" t="s">
+        <v>118</v>
+      </c>
+      <c r="E58" t="s">
         <v>119</v>
-      </c>
-      <c r="E58" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B59">
         <v>3</v>
       </c>
       <c r="D59" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E59" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F59" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B60">
         <v>3</v>
       </c>
       <c r="D60" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E60" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F60" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B61">
         <v>3</v>
       </c>
       <c r="D61" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E61" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F61" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.2">
@@ -2988,10 +2985,10 @@
         <v>3</v>
       </c>
       <c r="D62" t="s">
+        <v>123</v>
+      </c>
+      <c r="E62" t="s">
         <v>124</v>
-      </c>
-      <c r="E62" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.2">
@@ -2999,10 +2996,10 @@
         <v>1</v>
       </c>
       <c r="C63" t="s">
+        <v>125</v>
+      </c>
+      <c r="D63" t="s">
         <v>126</v>
-      </c>
-      <c r="D63" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.2">
@@ -3010,61 +3007,61 @@
         <v>2</v>
       </c>
       <c r="C64" t="s">
+        <v>127</v>
+      </c>
+      <c r="E64" t="s">
         <v>128</v>
-      </c>
-      <c r="E64" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B65">
         <v>3</v>
       </c>
       <c r="D65" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E65" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F65" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B66">
         <v>3</v>
       </c>
       <c r="D66" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E66" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F66" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B67">
         <v>3</v>
       </c>
       <c r="D67" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E67" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F67" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.2">
@@ -3072,10 +3069,10 @@
         <v>3</v>
       </c>
       <c r="D68" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E68" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.2">
@@ -3083,44 +3080,44 @@
         <v>2</v>
       </c>
       <c r="C69" t="s">
+        <v>133</v>
+      </c>
+      <c r="E69" t="s">
         <v>134</v>
-      </c>
-      <c r="E69" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B70">
         <v>3</v>
       </c>
       <c r="D70" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E70" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F70" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B71">
         <v>3</v>
       </c>
       <c r="D71" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E71" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F71" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.2">
@@ -3128,44 +3125,44 @@
         <v>2</v>
       </c>
       <c r="C72" t="s">
+        <v>137</v>
+      </c>
+      <c r="E72" t="s">
         <v>138</v>
-      </c>
-      <c r="E72" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B73">
         <v>3</v>
       </c>
       <c r="D73" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E73" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F73" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B74">
         <v>3</v>
       </c>
       <c r="D74" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E74" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F74" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.2">
@@ -3173,61 +3170,61 @@
         <v>2</v>
       </c>
       <c r="C75" t="s">
+        <v>141</v>
+      </c>
+      <c r="E75" t="s">
         <v>142</v>
-      </c>
-      <c r="E75" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B76">
         <v>3</v>
       </c>
       <c r="D76" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E76" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F76" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B77">
         <v>3</v>
       </c>
       <c r="D77" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E77" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F77" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B78">
         <v>3</v>
       </c>
       <c r="D78" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E78" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F78" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.2">
@@ -3235,10 +3232,10 @@
         <v>1</v>
       </c>
       <c r="C79" t="s">
+        <v>146</v>
+      </c>
+      <c r="D79" t="s">
         <v>147</v>
-      </c>
-      <c r="D79" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.2">
@@ -3246,10 +3243,10 @@
         <v>2</v>
       </c>
       <c r="C80" t="s">
+        <v>148</v>
+      </c>
+      <c r="E80" t="s">
         <v>149</v>
-      </c>
-      <c r="E80" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.2">
@@ -3257,61 +3254,61 @@
         <v>3</v>
       </c>
       <c r="C81" t="s">
+        <v>150</v>
+      </c>
+      <c r="E81" t="s">
         <v>151</v>
-      </c>
-      <c r="E81" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B82">
         <v>4</v>
       </c>
       <c r="D82" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E82" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F82" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B83">
         <v>4</v>
       </c>
       <c r="D83" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E83" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F83" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B84">
         <v>4</v>
       </c>
       <c r="D84" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E84" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F84" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.2">
@@ -3319,78 +3316,78 @@
         <v>3</v>
       </c>
       <c r="C85" t="s">
+        <v>155</v>
+      </c>
+      <c r="E85" t="s">
         <v>156</v>
-      </c>
-      <c r="E85" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B86">
         <v>4</v>
       </c>
       <c r="D86" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E86" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F86" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B87">
         <v>4</v>
       </c>
       <c r="D87" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E87" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F87" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B88">
         <v>4</v>
       </c>
       <c r="D88" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E88" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F88" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B89">
         <v>4</v>
       </c>
       <c r="D89" t="s">
+        <v>160</v>
+      </c>
+      <c r="E89" t="s">
         <v>161</v>
       </c>
-      <c r="E89" t="s">
+      <c r="F89" t="s">
         <v>162</v>
-      </c>
-      <c r="F89" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.2">
@@ -3398,44 +3395,44 @@
         <v>3</v>
       </c>
       <c r="C90" t="s">
+        <v>163</v>
+      </c>
+      <c r="E90" t="s">
         <v>164</v>
-      </c>
-      <c r="E90" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B91">
         <v>4</v>
       </c>
       <c r="D91" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E91" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F91" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B92">
         <v>4</v>
       </c>
       <c r="D92" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E92" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F92" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.2">
@@ -3443,10 +3440,10 @@
         <v>2</v>
       </c>
       <c r="C93" t="s">
+        <v>167</v>
+      </c>
+      <c r="E93" t="s">
         <v>168</v>
-      </c>
-      <c r="E93" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.2">
@@ -3454,78 +3451,78 @@
         <v>3</v>
       </c>
       <c r="C94" t="s">
+        <v>169</v>
+      </c>
+      <c r="E94" t="s">
         <v>170</v>
-      </c>
-      <c r="E94" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B95">
         <v>4</v>
       </c>
       <c r="D95" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E95" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F95" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B96">
         <v>4</v>
       </c>
       <c r="D96" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E96" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F96" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B97">
         <v>4</v>
       </c>
       <c r="D97" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E97" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F97" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B98">
         <v>4</v>
       </c>
       <c r="D98" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E98" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F98" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.2">
@@ -3533,10 +3530,10 @@
         <v>4</v>
       </c>
       <c r="D99" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E99" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.2">
@@ -3544,10 +3541,10 @@
         <v>1</v>
       </c>
       <c r="C100" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D100" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.2">
@@ -3555,10 +3552,10 @@
         <v>2</v>
       </c>
       <c r="C101" t="s">
+        <v>177</v>
+      </c>
+      <c r="E101" t="s">
         <v>178</v>
-      </c>
-      <c r="E101" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.2">
@@ -3566,61 +3563,61 @@
         <v>3</v>
       </c>
       <c r="C102" t="s">
+        <v>179</v>
+      </c>
+      <c r="E102" t="s">
         <v>180</v>
-      </c>
-      <c r="E102" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B103">
         <v>4</v>
       </c>
       <c r="D103" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E103" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F103" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B104">
         <v>4</v>
       </c>
       <c r="D104" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E104" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F104" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B105">
         <v>4</v>
       </c>
       <c r="D105" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E105" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F105" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.2">
@@ -3628,78 +3625,78 @@
         <v>3</v>
       </c>
       <c r="C106" t="s">
+        <v>184</v>
+      </c>
+      <c r="E106" t="s">
         <v>185</v>
-      </c>
-      <c r="E106" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B107">
         <v>4</v>
       </c>
       <c r="D107" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E107" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F107" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B108">
         <v>4</v>
       </c>
       <c r="D108" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E108" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="F108" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B109">
         <v>4</v>
       </c>
       <c r="D109" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E109" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F109" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B110">
         <v>4</v>
       </c>
       <c r="D110" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E110" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F110" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.2">
@@ -3707,10 +3704,10 @@
         <v>2</v>
       </c>
       <c r="C111" t="s">
+        <v>190</v>
+      </c>
+      <c r="E111" t="s">
         <v>191</v>
-      </c>
-      <c r="E111" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.2">
@@ -3718,61 +3715,61 @@
         <v>3</v>
       </c>
       <c r="C112" t="s">
+        <v>192</v>
+      </c>
+      <c r="E112" t="s">
         <v>193</v>
-      </c>
-      <c r="E112" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B113">
         <v>4</v>
       </c>
       <c r="D113" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E113" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F113" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B114">
         <v>4</v>
       </c>
       <c r="D114" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E114" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F114" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B115">
         <v>4</v>
       </c>
       <c r="D115" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E115" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F115" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.2">
@@ -3780,44 +3777,44 @@
         <v>3</v>
       </c>
       <c r="C116" t="s">
+        <v>197</v>
+      </c>
+      <c r="E116" t="s">
         <v>198</v>
-      </c>
-      <c r="E116" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B117">
         <v>4</v>
       </c>
       <c r="D117" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E117" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F117" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B118">
         <v>4</v>
       </c>
       <c r="D118" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E118" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F118" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.2">
@@ -3825,44 +3822,44 @@
         <v>3</v>
       </c>
       <c r="C119" t="s">
+        <v>201</v>
+      </c>
+      <c r="E119" t="s">
         <v>202</v>
-      </c>
-      <c r="E119" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B120">
         <v>4</v>
       </c>
       <c r="D120" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E120" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="F120" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B121">
         <v>4</v>
       </c>
       <c r="D121" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E121" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F121" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.2">
@@ -3870,78 +3867,78 @@
         <v>3</v>
       </c>
       <c r="C122" t="s">
+        <v>205</v>
+      </c>
+      <c r="E122" t="s">
         <v>206</v>
-      </c>
-      <c r="E122" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B123">
         <v>4</v>
       </c>
       <c r="D123" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E123" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F123" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B124">
         <v>4</v>
       </c>
       <c r="D124" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E124" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F124" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B125">
         <v>4</v>
       </c>
       <c r="D125" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E125" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F125" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B126">
         <v>4</v>
       </c>
       <c r="D126" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E126" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F126" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.2">
@@ -3949,44 +3946,44 @@
         <v>3</v>
       </c>
       <c r="C127" t="s">
+        <v>211</v>
+      </c>
+      <c r="E127" t="s">
         <v>212</v>
-      </c>
-      <c r="E127" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B128">
         <v>4</v>
       </c>
       <c r="D128" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E128" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F128" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B129">
         <v>4</v>
       </c>
       <c r="D129" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E129" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F129" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.2">
@@ -3994,44 +3991,44 @@
         <v>3</v>
       </c>
       <c r="C130" t="s">
+        <v>215</v>
+      </c>
+      <c r="E130" t="s">
         <v>216</v>
-      </c>
-      <c r="E130" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B131">
         <v>4</v>
       </c>
       <c r="D131" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E131" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F131" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B132">
         <v>4</v>
       </c>
       <c r="D132" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E132" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F132" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.2">
@@ -4039,61 +4036,61 @@
         <v>3</v>
       </c>
       <c r="C133" t="s">
+        <v>219</v>
+      </c>
+      <c r="E133" t="s">
         <v>220</v>
-      </c>
-      <c r="E133" t="s">
-        <v>221</v>
       </c>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B134">
         <v>4</v>
       </c>
       <c r="D134" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E134" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F134" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B135">
         <v>4</v>
       </c>
       <c r="D135" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E135" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="F135" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B136">
         <v>4</v>
       </c>
       <c r="D136" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E136" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="F136" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.2">
@@ -4101,10 +4098,10 @@
         <v>2</v>
       </c>
       <c r="C137" t="s">
+        <v>224</v>
+      </c>
+      <c r="E137" t="s">
         <v>225</v>
-      </c>
-      <c r="E137" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.2">
@@ -4112,44 +4109,44 @@
         <v>3</v>
       </c>
       <c r="C138" t="s">
+        <v>226</v>
+      </c>
+      <c r="E138" t="s">
         <v>227</v>
-      </c>
-      <c r="E138" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B139">
         <v>4</v>
       </c>
       <c r="D139" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E139" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F139" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B140">
         <v>4</v>
       </c>
       <c r="D140" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E140" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F140" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.2">
@@ -4157,61 +4154,61 @@
         <v>3</v>
       </c>
       <c r="C141" t="s">
+        <v>230</v>
+      </c>
+      <c r="E141" t="s">
         <v>231</v>
-      </c>
-      <c r="E141" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B142">
         <v>4</v>
       </c>
       <c r="D142" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E142" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F142" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B143">
         <v>4</v>
       </c>
       <c r="D143" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E143" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F143" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B144">
         <v>4</v>
       </c>
       <c r="D144" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E144" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F144" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.2">
@@ -4219,44 +4216,44 @@
         <v>3</v>
       </c>
       <c r="C145" t="s">
+        <v>235</v>
+      </c>
+      <c r="E145" t="s">
         <v>236</v>
-      </c>
-      <c r="E145" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B146">
         <v>4</v>
       </c>
       <c r="D146" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E146" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F146" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B147">
         <v>4</v>
       </c>
       <c r="D147" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E147" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F147" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.2">
@@ -4264,44 +4261,44 @@
         <v>3</v>
       </c>
       <c r="C148" t="s">
+        <v>239</v>
+      </c>
+      <c r="E148" t="s">
         <v>240</v>
-      </c>
-      <c r="E148" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B149">
         <v>4</v>
       </c>
       <c r="D149" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E149" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="F149" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B150">
         <v>4</v>
       </c>
       <c r="D150" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E150" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="F150" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="151" spans="1:6" x14ac:dyDescent="0.2">
@@ -4309,10 +4306,10 @@
         <v>1</v>
       </c>
       <c r="C151" t="s">
+        <v>243</v>
+      </c>
+      <c r="D151" t="s">
         <v>244</v>
-      </c>
-      <c r="D151" t="s">
-        <v>245</v>
       </c>
     </row>
     <row r="152" spans="1:6" x14ac:dyDescent="0.2">
@@ -4320,61 +4317,61 @@
         <v>2</v>
       </c>
       <c r="C152" t="s">
+        <v>245</v>
+      </c>
+      <c r="E152" t="s">
         <v>246</v>
-      </c>
-      <c r="E152" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="153" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B153">
         <v>3</v>
       </c>
       <c r="D153" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E153" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F153" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="154" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B154">
         <v>3</v>
       </c>
       <c r="D154" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E154" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="F154" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="155" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B155">
         <v>3</v>
       </c>
       <c r="D155" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E155" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F155" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="156" spans="1:6" x14ac:dyDescent="0.2">
@@ -4382,10 +4379,10 @@
         <v>3</v>
       </c>
       <c r="D156" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E156" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="157" spans="1:6" x14ac:dyDescent="0.2">
@@ -4393,44 +4390,44 @@
         <v>2</v>
       </c>
       <c r="C157" t="s">
+        <v>251</v>
+      </c>
+      <c r="E157" t="s">
         <v>252</v>
-      </c>
-      <c r="E157" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="158" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B158">
         <v>3</v>
       </c>
       <c r="D158" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E158" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="F158" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="159" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B159">
         <v>3</v>
       </c>
       <c r="D159" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E159" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="F159" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="160" spans="1:6" x14ac:dyDescent="0.2">
@@ -4438,10 +4435,10 @@
         <v>1</v>
       </c>
       <c r="C160" t="s">
+        <v>255</v>
+      </c>
+      <c r="D160" t="s">
         <v>256</v>
-      </c>
-      <c r="D160" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.2">
@@ -4449,44 +4446,44 @@
         <v>2</v>
       </c>
       <c r="C161" t="s">
+        <v>257</v>
+      </c>
+      <c r="E161" t="s">
         <v>258</v>
-      </c>
-      <c r="E161" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="162" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B162">
         <v>3</v>
       </c>
       <c r="D162" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E162" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F162" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="163" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B163">
         <v>3</v>
       </c>
       <c r="D163" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E163" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="F163" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="164" spans="1:6" x14ac:dyDescent="0.2">
@@ -4494,27 +4491,27 @@
         <v>2</v>
       </c>
       <c r="C164" t="s">
+        <v>261</v>
+      </c>
+      <c r="E164" t="s">
         <v>262</v>
-      </c>
-      <c r="E164" t="s">
-        <v>263</v>
       </c>
     </row>
     <row r="165" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B165">
         <v>3</v>
       </c>
       <c r="D165" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E165" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F165" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="166" spans="1:6" x14ac:dyDescent="0.2">
@@ -4522,10 +4519,10 @@
         <v>1</v>
       </c>
       <c r="C166" t="s">
+        <v>264</v>
+      </c>
+      <c r="D166" t="s">
         <v>265</v>
-      </c>
-      <c r="D166" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="167" spans="1:6" x14ac:dyDescent="0.2">
@@ -4533,10 +4530,10 @@
         <v>2</v>
       </c>
       <c r="C167" t="s">
+        <v>266</v>
+      </c>
+      <c r="E167" t="s">
         <v>267</v>
-      </c>
-      <c r="E167" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="168" spans="1:6" x14ac:dyDescent="0.2">
@@ -4544,44 +4541,44 @@
         <v>3</v>
       </c>
       <c r="C168" t="s">
+        <v>268</v>
+      </c>
+      <c r="E168" t="s">
         <v>269</v>
-      </c>
-      <c r="E168" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="169" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A169" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B169">
         <v>4</v>
       </c>
       <c r="D169" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E169" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="F169" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="170" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A170" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B170">
         <v>4</v>
       </c>
       <c r="D170" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E170" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F170" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="171" spans="1:6" x14ac:dyDescent="0.2">
@@ -4589,44 +4586,44 @@
         <v>3</v>
       </c>
       <c r="C171" t="s">
+        <v>272</v>
+      </c>
+      <c r="E171" t="s">
         <v>273</v>
-      </c>
-      <c r="E171" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="172" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A172" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B172">
         <v>4</v>
       </c>
       <c r="D172" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E172" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F172" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="173" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A173" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B173">
         <v>4</v>
       </c>
       <c r="D173" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E173" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F173" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="174" spans="1:6" x14ac:dyDescent="0.2">
@@ -4634,44 +4631,44 @@
         <v>3</v>
       </c>
       <c r="C174" t="s">
+        <v>276</v>
+      </c>
+      <c r="E174" t="s">
         <v>277</v>
-      </c>
-      <c r="E174" t="s">
-        <v>278</v>
       </c>
     </row>
     <row r="175" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A175" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B175">
         <v>4</v>
       </c>
       <c r="D175" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E175" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F175" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="176" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B176">
         <v>4</v>
       </c>
       <c r="D176" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E176" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F176" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="177" spans="1:6" x14ac:dyDescent="0.2">
@@ -4679,61 +4676,61 @@
         <v>3</v>
       </c>
       <c r="C177" t="s">
+        <v>280</v>
+      </c>
+      <c r="E177" t="s">
         <v>281</v>
-      </c>
-      <c r="E177" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="178" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B178">
         <v>4</v>
       </c>
       <c r="D178" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E178" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="F178" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="179" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B179">
         <v>4</v>
       </c>
       <c r="D179" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E179" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F179" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="180" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B180">
         <v>4</v>
       </c>
       <c r="D180" t="s">
+        <v>284</v>
+      </c>
+      <c r="E180" t="s">
         <v>285</v>
       </c>
-      <c r="E180" t="s">
+      <c r="F180" t="s">
         <v>286</v>
-      </c>
-      <c r="F180" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="181" spans="1:6" x14ac:dyDescent="0.2">
@@ -4741,44 +4738,44 @@
         <v>3</v>
       </c>
       <c r="C181" t="s">
+        <v>287</v>
+      </c>
+      <c r="E181" t="s">
         <v>288</v>
-      </c>
-      <c r="E181" t="s">
-        <v>289</v>
       </c>
     </row>
     <row r="182" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A182" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B182">
         <v>4</v>
       </c>
       <c r="D182" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E182" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="F182" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="183" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B183">
         <v>4</v>
       </c>
       <c r="D183" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="E183" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="F183" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="184" spans="1:6" x14ac:dyDescent="0.2">
@@ -4786,27 +4783,27 @@
         <v>3</v>
       </c>
       <c r="C184" t="s">
+        <v>291</v>
+      </c>
+      <c r="E184" t="s">
         <v>292</v>
-      </c>
-      <c r="E184" t="s">
-        <v>293</v>
       </c>
     </row>
     <row r="185" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A185" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B185">
         <v>4</v>
       </c>
       <c r="D185" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E185" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F185" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="186" spans="1:6" x14ac:dyDescent="0.2">
@@ -4814,27 +4811,27 @@
         <v>3</v>
       </c>
       <c r="C186" t="s">
+        <v>294</v>
+      </c>
+      <c r="E186" t="s">
         <v>295</v>
-      </c>
-      <c r="E186" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="187" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A187" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B187">
         <v>4</v>
       </c>
       <c r="D187" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E187" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F187" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="188" spans="1:6" x14ac:dyDescent="0.2">
@@ -4842,44 +4839,44 @@
         <v>3</v>
       </c>
       <c r="C188" t="s">
+        <v>297</v>
+      </c>
+      <c r="E188" t="s">
         <v>298</v>
-      </c>
-      <c r="E188" t="s">
-        <v>299</v>
       </c>
     </row>
     <row r="189" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A189" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B189">
         <v>4</v>
       </c>
       <c r="D189" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E189" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="F189" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="190" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A190" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B190">
         <v>4</v>
       </c>
       <c r="D190" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="E190" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="F190" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="191" spans="1:6" x14ac:dyDescent="0.2">
@@ -4887,10 +4884,10 @@
         <v>2</v>
       </c>
       <c r="C191" t="s">
+        <v>301</v>
+      </c>
+      <c r="E191" t="s">
         <v>302</v>
-      </c>
-      <c r="E191" t="s">
-        <v>303</v>
       </c>
     </row>
     <row r="192" spans="1:6" x14ac:dyDescent="0.2">
@@ -4898,27 +4895,27 @@
         <v>3</v>
       </c>
       <c r="C192" t="s">
+        <v>303</v>
+      </c>
+      <c r="E192" t="s">
         <v>304</v>
-      </c>
-      <c r="E192" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="193" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A193" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B193">
         <v>4</v>
       </c>
       <c r="D193" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E193" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="F193" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="194" spans="1:6" x14ac:dyDescent="0.2">
@@ -4926,27 +4923,27 @@
         <v>3</v>
       </c>
       <c r="C194" t="s">
+        <v>306</v>
+      </c>
+      <c r="E194" t="s">
         <v>307</v>
-      </c>
-      <c r="E194" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="195" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A195" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B195">
         <v>4</v>
       </c>
       <c r="D195" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E195" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="F195" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="196" spans="1:6" x14ac:dyDescent="0.2">
@@ -4954,27 +4951,27 @@
         <v>3</v>
       </c>
       <c r="C196" t="s">
+        <v>309</v>
+      </c>
+      <c r="E196" t="s">
         <v>310</v>
-      </c>
-      <c r="E196" t="s">
-        <v>311</v>
       </c>
     </row>
     <row r="197" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A197" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B197">
         <v>4</v>
       </c>
       <c r="D197" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E197" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="F197" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="198" spans="1:6" x14ac:dyDescent="0.2">
@@ -4982,27 +4979,27 @@
         <v>3</v>
       </c>
       <c r="C198" t="s">
+        <v>312</v>
+      </c>
+      <c r="E198" t="s">
         <v>313</v>
-      </c>
-      <c r="E198" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="199" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A199" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B199">
         <v>4</v>
       </c>
       <c r="D199" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E199" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F199" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="200" spans="1:6" x14ac:dyDescent="0.2">
@@ -5010,27 +5007,27 @@
         <v>3</v>
       </c>
       <c r="C200" t="s">
+        <v>315</v>
+      </c>
+      <c r="E200" t="s">
         <v>316</v>
-      </c>
-      <c r="E200" t="s">
-        <v>317</v>
       </c>
     </row>
     <row r="201" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A201" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B201">
         <v>4</v>
       </c>
       <c r="D201" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E201" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="F201" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="202" spans="1:6" x14ac:dyDescent="0.2">
@@ -5038,27 +5035,27 @@
         <v>3</v>
       </c>
       <c r="C202" t="s">
+        <v>318</v>
+      </c>
+      <c r="E202" t="s">
         <v>319</v>
-      </c>
-      <c r="E202" t="s">
-        <v>320</v>
       </c>
     </row>
     <row r="203" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A203" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B203">
         <v>4</v>
       </c>
       <c r="D203" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E203" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F203" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="204" spans="1:6" x14ac:dyDescent="0.2">
@@ -5066,27 +5063,27 @@
         <v>3</v>
       </c>
       <c r="C204" t="s">
+        <v>321</v>
+      </c>
+      <c r="E204" t="s">
         <v>322</v>
-      </c>
-      <c r="E204" t="s">
-        <v>323</v>
       </c>
     </row>
     <row r="205" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A205" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B205">
         <v>4</v>
       </c>
       <c r="D205" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E205" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="F205" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="206" spans="1:6" x14ac:dyDescent="0.2">
@@ -5094,10 +5091,10 @@
         <v>2</v>
       </c>
       <c r="C206" t="s">
+        <v>324</v>
+      </c>
+      <c r="E206" t="s">
         <v>325</v>
-      </c>
-      <c r="E206" t="s">
-        <v>326</v>
       </c>
     </row>
     <row r="207" spans="1:6" x14ac:dyDescent="0.2">
@@ -5105,27 +5102,27 @@
         <v>3</v>
       </c>
       <c r="C207" t="s">
+        <v>326</v>
+      </c>
+      <c r="E207" t="s">
         <v>327</v>
-      </c>
-      <c r="E207" t="s">
-        <v>328</v>
       </c>
     </row>
     <row r="208" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A208" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B208">
         <v>4</v>
       </c>
       <c r="D208" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E208" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="F208" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="209" spans="1:6" x14ac:dyDescent="0.2">
@@ -5133,27 +5130,27 @@
         <v>3</v>
       </c>
       <c r="C209" t="s">
+        <v>329</v>
+      </c>
+      <c r="E209" t="s">
         <v>330</v>
-      </c>
-      <c r="E209" t="s">
-        <v>331</v>
       </c>
     </row>
     <row r="210" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A210" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B210">
         <v>4</v>
       </c>
       <c r="D210" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E210" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F210" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="211" spans="1:6" x14ac:dyDescent="0.2">
@@ -5161,10 +5158,10 @@
         <v>2</v>
       </c>
       <c r="C211" t="s">
+        <v>332</v>
+      </c>
+      <c r="E211" t="s">
         <v>333</v>
-      </c>
-      <c r="E211" t="s">
-        <v>334</v>
       </c>
     </row>
     <row r="212" spans="1:6" x14ac:dyDescent="0.2">
@@ -5172,27 +5169,27 @@
         <v>3</v>
       </c>
       <c r="C212" t="s">
+        <v>334</v>
+      </c>
+      <c r="E212" t="s">
         <v>335</v>
-      </c>
-      <c r="E212" t="s">
-        <v>336</v>
       </c>
     </row>
     <row r="213" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A213" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B213">
         <v>4</v>
       </c>
       <c r="D213" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E213" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F213" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="214" spans="1:6" x14ac:dyDescent="0.2">
@@ -5200,27 +5197,27 @@
         <v>3</v>
       </c>
       <c r="C214" t="s">
+        <v>337</v>
+      </c>
+      <c r="E214" t="s">
         <v>338</v>
-      </c>
-      <c r="E214" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="215" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A215" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B215">
         <v>4</v>
       </c>
       <c r="D215" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E215" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="F215" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="216" spans="1:6" x14ac:dyDescent="0.2">
@@ -5228,27 +5225,27 @@
         <v>3</v>
       </c>
       <c r="C216" t="s">
+        <v>340</v>
+      </c>
+      <c r="E216" t="s">
         <v>341</v>
-      </c>
-      <c r="E216" t="s">
-        <v>342</v>
       </c>
     </row>
     <row r="217" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A217" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B217">
         <v>4</v>
       </c>
       <c r="D217" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E217" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="F217" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="218" spans="1:6" x14ac:dyDescent="0.2">
@@ -5256,10 +5253,10 @@
         <v>2</v>
       </c>
       <c r="C218" t="s">
+        <v>343</v>
+      </c>
+      <c r="E218" t="s">
         <v>344</v>
-      </c>
-      <c r="E218" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="219" spans="1:6" x14ac:dyDescent="0.2">
@@ -5267,27 +5264,27 @@
         <v>3</v>
       </c>
       <c r="C219" t="s">
+        <v>345</v>
+      </c>
+      <c r="E219" t="s">
         <v>346</v>
-      </c>
-      <c r="E219" t="s">
-        <v>347</v>
       </c>
     </row>
     <row r="220" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A220" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B220">
         <v>4</v>
       </c>
       <c r="D220" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E220" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="F220" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="221" spans="1:6" x14ac:dyDescent="0.2">
@@ -5295,27 +5292,27 @@
         <v>3</v>
       </c>
       <c r="C221" t="s">
+        <v>348</v>
+      </c>
+      <c r="E221" t="s">
         <v>349</v>
-      </c>
-      <c r="E221" t="s">
-        <v>350</v>
       </c>
     </row>
     <row r="222" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A222" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B222">
         <v>4</v>
       </c>
       <c r="D222" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E222" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="F222" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="223" spans="1:6" x14ac:dyDescent="0.2">
@@ -5323,10 +5320,10 @@
         <v>1</v>
       </c>
       <c r="C223" t="s">
+        <v>351</v>
+      </c>
+      <c r="D223" t="s">
         <v>352</v>
-      </c>
-      <c r="D223" t="s">
-        <v>353</v>
       </c>
     </row>
     <row r="224" spans="1:6" x14ac:dyDescent="0.2">
@@ -5334,27 +5331,27 @@
         <v>2</v>
       </c>
       <c r="C224" t="s">
+        <v>353</v>
+      </c>
+      <c r="E224" t="s">
         <v>354</v>
-      </c>
-      <c r="E224" t="s">
-        <v>355</v>
       </c>
     </row>
     <row r="225" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A225" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B225">
         <v>3</v>
       </c>
       <c r="D225" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E225" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="F225" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="226" spans="1:6" x14ac:dyDescent="0.2">
@@ -5362,27 +5359,27 @@
         <v>2</v>
       </c>
       <c r="C226" t="s">
+        <v>356</v>
+      </c>
+      <c r="E226" t="s">
         <v>357</v>
-      </c>
-      <c r="E226" t="s">
-        <v>358</v>
       </c>
     </row>
     <row r="227" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A227" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B227">
         <v>3</v>
       </c>
       <c r="D227" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E227" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="F227" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="228" spans="1:6" x14ac:dyDescent="0.2">
@@ -5390,27 +5387,27 @@
         <v>2</v>
       </c>
       <c r="C228" t="s">
+        <v>359</v>
+      </c>
+      <c r="E228" t="s">
         <v>360</v>
-      </c>
-      <c r="E228" t="s">
-        <v>361</v>
       </c>
     </row>
     <row r="229" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A229" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B229">
         <v>3</v>
       </c>
       <c r="D229" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E229" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="F229" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="230" spans="1:6" x14ac:dyDescent="0.2">
@@ -5418,27 +5415,27 @@
         <v>2</v>
       </c>
       <c r="C230" t="s">
+        <v>362</v>
+      </c>
+      <c r="E230" t="s">
         <v>363</v>
-      </c>
-      <c r="E230" t="s">
-        <v>364</v>
       </c>
     </row>
     <row r="231" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A231" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B231">
         <v>3</v>
       </c>
       <c r="D231" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E231" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="F231" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -5456,7 +5453,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -5464,7 +5461,7 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -5479,13 +5476,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B1" t="s">
         <v>10</v>
       </c>
       <c r="C1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -5493,10 +5490,10 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
+        <v>366</v>
+      </c>
+      <c r="C2" t="s">
         <v>367</v>
-      </c>
-      <c r="C2" t="s">
-        <v>368</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -5504,10 +5501,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
+        <v>368</v>
+      </c>
+      <c r="C3" t="s">
         <v>369</v>
-      </c>
-      <c r="C3" t="s">
-        <v>370</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -5515,10 +5512,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
+        <v>370</v>
+      </c>
+      <c r="C4" t="s">
         <v>371</v>
-      </c>
-      <c r="C4" t="s">
-        <v>372</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -5526,10 +5523,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
+        <v>372</v>
+      </c>
+      <c r="C5" t="s">
         <v>373</v>
-      </c>
-      <c r="C5" t="s">
-        <v>374</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -5537,10 +5534,10 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
+        <v>374</v>
+      </c>
+      <c r="C6" t="s">
         <v>375</v>
-      </c>
-      <c r="C6" t="s">
-        <v>376</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
@@ -5548,10 +5545,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
+        <v>376</v>
+      </c>
+      <c r="C7" t="s">
         <v>377</v>
-      </c>
-      <c r="C7" t="s">
-        <v>378</v>
       </c>
     </row>
   </sheetData>
@@ -5569,7 +5566,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -5577,7 +5574,7 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -5598,73 +5595,73 @@
         <v>10</v>
       </c>
       <c r="C1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B2" t="s">
+        <v>378</v>
+      </c>
+      <c r="C2" t="s">
         <v>379</v>
-      </c>
-      <c r="C2" t="s">
-        <v>380</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B3" t="s">
+        <v>380</v>
+      </c>
+      <c r="C3" t="s">
         <v>381</v>
-      </c>
-      <c r="C3" t="s">
-        <v>382</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B4" t="s">
+        <v>382</v>
+      </c>
+      <c r="C4" t="s">
         <v>383</v>
-      </c>
-      <c r="C4" t="s">
-        <v>384</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B5" t="s">
+        <v>384</v>
+      </c>
+      <c r="C5" t="s">
         <v>385</v>
-      </c>
-      <c r="C5" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>386</v>
+      </c>
+      <c r="B6" t="s">
         <v>387</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>388</v>
-      </c>
-      <c r="C6" t="s">
-        <v>389</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B7" t="s">
+        <v>389</v>
+      </c>
+      <c r="C7" t="s">
         <v>390</v>
-      </c>
-      <c r="C7" t="s">
-        <v>391</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add tisax in name to facilitate search
</commit_message>
<xml_diff>
--- a/tools/excel/tisax/tisax-v5.1.xlsx
+++ b/tools/excel/tisax/tisax-v5.1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericlaubacher/Documents/GitHub/ciso-assistant-community/tools/excel/tisax/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F853DD6F-D3E8-E648-AF53-C783D517EFAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A975B86A-C31A-A541-8D19-1D12D14C7742}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="library_meta" sheetId="1" r:id="rId1"/>
@@ -1561,17 +1561,24 @@
     <t>Protects physical prototypes which are classified as requiring protection. Prototypes include vehicles, components and parts. The owner of the intellectual property for the prototype is considered the owner of the prototype. The owner's commissioning department is responsible for classifying the protection need of a prototype. For prototypes classified as requiring high or very high protection, the minimum requirements for prototype protection must be applied.</t>
   </si>
   <si>
-    <t>Trusted Information Security Assessment Exchange v5.1</t>
+    <t>Trusted Information Security Assessment Exchange (TISAX) v5.1</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1597,8 +1604,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1903,6 +1911,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="255.83203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -1993,6 +2004,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="255.83203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -2030,7 +2044,7 @@
       <c r="A5" t="s">
         <v>10</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="1" t="s">
         <v>391</v>
       </c>
     </row>

</xml_diff>